<commit_message>
State unaudited/not-GAAP in the reserve plan; statements issued twice a year
- generate_entity_workbooks.py: Instructions and Fund Summary say the plan
  is unaudited planning estimates, not a financial statement, not
  prepared under U.S. GAAP, and not a CAI reserve study. Condo IV
  workbook regenerated (figures unchanged)
- Condo IV statement: Background says it is issued twice a year
  (mid-year in the fall with the proposed budget, full-year in the
  spring); this is the mid-year 2026 edition
- Entity_Statement_Prompt_Instructions.md: new section 0 with the
  twice-a-year schedule and what changes per edition
</commit_message>
<xml_diff>
--- a/Condo_IV_Reserve_Plan.xlsx
+++ b/Condo_IV_Reserve_Plan.xlsx
@@ -47,18 +47,18 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00666666"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -165,34 +165,34 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -964,7 +964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E82"/>
+  <dimension ref="B1:E83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -988,584 +988,591 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="B4" s="2" t="inlineStr">
+    <row r="3">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Unaudited planning estimates. This plan is not a financial statement, is not prepared in accordance with U.S. GAAP, and is not a reserve study under the CAI National Reserve Study Standards. Future costs, timing and balances are estimates and will differ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>How to read this workbook</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="B5" s="3" t="inlineStr">
+    <row r="6">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>START on the 'Fund Summary' tab — it shows the three funds, their targets/floors, the</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="B6" s="3" t="inlineStr">
+    <row r="7">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>per-unit monthly funding, and the 'Reserve Funding Status' all on one page.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="B7" s="3" t="inlineStr">
+    <row r="8">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>The three fund tabs — Emergency Reserve, Long-Term Maintenance, Operating Reserve — each</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="B8" s="3" t="inlineStr">
+    <row r="9">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>show that fund's year-by-year balance from 2027 to 2050.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" s="3" t="inlineStr">
+    <row r="10">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>'Components' lists every capital item and its cost; 'Expenditure Chart' plots spending by year.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="B10" s="3" t="inlineStr">
+    <row r="11">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Yellow cells are inputs you can edit; every other cell is calculated automatically.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="4" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Data Sources:</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="3" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Based on Becht Engineering Capital Reserve Study (Project 25-1140, February 2026)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="3" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Entity allocations derived from Falcon Group Report (2022) per-entity quantity ratios</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="2" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>Overview</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="3" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Number of units: 98</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="3" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Total replacement cost (current dollars): $3,594,809</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="3" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Total reserve cash to allocate (projected reserve cash at 12/31/2026 (from the 2027 budget)): $176,604</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="3" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Fund contributions are solved automatically (see Fund Summary) and are fully editable.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="3" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Planning horizon: 2027-2050 (24 years)</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="2" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Funding Model Assumptions</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="3" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>Annual contributions grow at a configurable rate (default 3%) to keep pace with inflation.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="3" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Reserve funds earn interest at a configurable rate (default 1%) annually.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="3" t="inlineStr">
+    <row r="27">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>Disbursements (expenditures) occur in the year projected by the Becht engineering study.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="3" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>All disbursement amounts include 3% annual inflation applied to current replacement costs.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="2" t="inlineStr">
+    <row r="30">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>Three-Fund Model</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="B30" s="3" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>This plan splits reserves into THREE decoupled funds, each with its own balance,</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="3" t="inlineStr">
+    <row r="32">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>annual contribution, floor, and monthly cost per unit. Each has its own tab.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="B32" s="3" t="inlineStr"/>
-    </row>
     <row r="33">
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>1. Emergency Reserve — self-funded buffer for uninsured structural &amp; shortfall exposure — deductible on HOA.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="3" t="inlineStr">
+    <row r="35">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">   Floor = a target you set (Fund Summary, yellow cell). Not drawn for routine work.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="B35" s="3" t="inlineStr">
+    <row r="36">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>2. Long-Term Maintenance — the Becht/Falcon capital replacement schedule.</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="B36" s="3" t="inlineStr">
+    <row r="37">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">   Floor = must NEVER drop below $0 in any year.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="B37" s="3" t="inlineStr">
+    <row r="38">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>3. Operating Reserve — decoupled buffer of operating expenses.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="B38" s="3" t="inlineStr">
+    <row r="39">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">   Floor = multiplier (1-3 months) x monthly operating expense, both set on Fund Summary.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="B39" s="3" t="inlineStr"/>
-    </row>
     <row r="40">
-      <c r="B40" s="3" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>Fund Summary sheet: set all inputs here (each fund's starting balance, target/floor and</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="B41" s="3" t="inlineStr">
+    <row r="42">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>contribution; unit count; growth; interest). Allocate current cash across the three funds'</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="B42" s="3" t="inlineStr">
+    <row r="43">
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>starting balances (Allocated Start column). Recommended: fund near-term Long-Term Maintenance</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="B43" s="3" t="inlineStr">
+    <row r="44">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>needs and Operating liquidity first, and build the Emergency Reserve from contributions.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="B44" s="3" t="inlineStr"/>
-    </row>
     <row r="45">
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>Percent Funded (Long-Term Maintenance) = reserve on hand / Fully Funded Balance. It is</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" s="3" t="inlineStr">
+    <row r="47">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>the industry (CAI) metric: under 30% = weak (high special-assessment risk), 30-70% = fair,</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="B47" s="3" t="inlineStr">
+    <row r="48">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>70%+ = strong.</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="B48" s="3" t="inlineStr"/>
-    </row>
     <row r="49">
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B49" s="4" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="B50" s="4" t="inlineStr">
         <is>
           <t>Reserve Funding Status — common charges should NOT be reduced until all three are Funded:</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="B50" s="3" t="inlineStr">
+    <row r="51">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  1 — Emergency Reserve is funded to its target.</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="B51" s="3" t="inlineStr">
+    <row r="52">
+      <c r="B52" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  2 — Long-Term Maintenance stays at/above $0 every year at the proposed contribution.</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="B52" s="3" t="inlineStr">
+    <row r="53">
+      <c r="B53" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  3 — Operating Reserve stays at/above its floor (multiplier x monthly operating expense).</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="B53" s="3" t="inlineStr">
+    <row r="54">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>The 'Reduction in common charges' cell says a reduction can be considered only when all three</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="B54" s="3" t="inlineStr">
+    <row r="55">
+      <c r="B55" s="4" t="inlineStr">
         <is>
           <t>are Funded. To model a reduction, lower a fund's Year-1 Contribution on the Fund Summary sheet.</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="B55" s="3" t="inlineStr">
+    <row r="56">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>Replace every yellow placeholder (targets, floors, total cash) with the entity's ACTUALS.</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="B57" s="2" t="inlineStr">
+    <row r="58">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>Components Covered by This Plan</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="B58" s="3" t="inlineStr">
+    <row r="59">
+      <c r="B59" s="4" t="inlineStr">
         <is>
           <t>See the 'Components' sheet for full detail. Summary:</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="B60" s="4" t="inlineStr">
+    <row r="61">
+      <c r="B61" s="5" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="C60" s="4" t="inlineStr">
+      <c r="C61" s="5" t="inlineStr">
         <is>
           <t>Allocated Cost</t>
         </is>
       </c>
-      <c r="D60" s="4" t="inlineStr">
+      <c r="D61" s="5" t="inlineStr">
         <is>
           <t>Replacement Year</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="B61" s="3" t="inlineStr">
+    <row r="62">
+      <c r="B62" s="4" t="inlineStr">
         <is>
           <t>Siding, Vinyl (Condo IV share)</t>
         </is>
       </c>
-      <c r="C61" s="5" t="n">
+      <c r="C62" s="6" t="n">
         <v>1651860</v>
       </c>
-      <c r="D61" s="3" t="n">
+      <c r="D62" s="4" t="n">
         <v>2049</v>
       </c>
     </row>
-    <row r="62">
-      <c r="B62" s="3" t="inlineStr">
+    <row r="63">
+      <c r="B63" s="4" t="inlineStr">
         <is>
           <t>Roof, Shingles - Townhouses (Condo IV share)</t>
         </is>
       </c>
-      <c r="C62" s="5" t="n">
+      <c r="C63" s="6" t="n">
         <v>880045</v>
       </c>
-      <c r="D62" s="3" t="n">
+      <c r="D63" s="4" t="n">
         <v>2050</v>
       </c>
     </row>
-    <row r="63">
-      <c r="B63" s="3" t="inlineStr">
+    <row r="64">
+      <c r="B64" s="4" t="inlineStr">
         <is>
           <t>Deck Framing &amp; Footings, Wood (Condo IV share)</t>
         </is>
       </c>
-      <c r="C63" s="5" t="n">
+      <c r="C64" s="6" t="n">
         <v>149760</v>
       </c>
-      <c r="D63" s="3" t="n">
+      <c r="D64" s="4" t="n">
         <v>2033</v>
       </c>
     </row>
-    <row r="64">
-      <c r="B64" s="3" t="inlineStr">
+    <row r="65">
+      <c r="B65" s="4" t="inlineStr">
         <is>
           <t>Deck Boards (surface), Wood (Condo IV share)</t>
         </is>
       </c>
-      <c r="C64" s="5" t="n">
+      <c r="C65" s="6" t="n">
         <v>131040</v>
       </c>
-      <c r="D64" s="3" t="n">
+      <c r="D65" s="4" t="n">
         <v>2033</v>
       </c>
     </row>
-    <row r="65">
-      <c r="B65" s="3" t="inlineStr">
+    <row r="66">
+      <c r="B66" s="4" t="inlineStr">
         <is>
           <t>Deck Railings &amp; Balusters, Wood (Condo IV share) (safety)</t>
         </is>
       </c>
-      <c r="C65" s="5" t="n">
+      <c r="C66" s="6" t="n">
         <v>93600</v>
       </c>
-      <c r="D65" s="3" t="n">
+      <c r="D66" s="4" t="n">
         <v>2033</v>
       </c>
     </row>
-    <row r="66">
-      <c r="B66" s="3" t="inlineStr">
+    <row r="67">
+      <c r="B67" s="4" t="inlineStr">
         <is>
           <t>Deck Railings — 2027 remaining replacements (5 rails)</t>
         </is>
       </c>
-      <c r="C66" s="5" t="n">
+      <c r="C67" s="6" t="n">
         <v>22500</v>
       </c>
-      <c r="D66" s="3" t="n">
+      <c r="D67" s="4" t="n">
         <v>2027</v>
       </c>
     </row>
-    <row r="67">
-      <c r="B67" s="3" t="inlineStr">
+    <row r="68">
+      <c r="B68" s="4" t="inlineStr">
         <is>
           <t>Deck Replacement, Composite (Condo IV share)</t>
         </is>
       </c>
-      <c r="C67" s="5" t="n">
+      <c r="C68" s="6" t="n">
         <v>132444</v>
       </c>
-      <c r="D67" s="3" t="n">
+      <c r="D68" s="4" t="n">
         <v>2053</v>
       </c>
     </row>
-    <row r="68">
-      <c r="B68" s="3" t="inlineStr">
+    <row r="69">
+      <c r="B69" s="4" t="inlineStr">
         <is>
           <t>Chimney Chase Covers (Condo IV share)</t>
         </is>
       </c>
-      <c r="C68" s="5" t="n">
+      <c r="C69" s="6" t="n">
         <v>125160</v>
       </c>
-      <c r="D68" s="3" t="n">
+      <c r="D69" s="4" t="n">
         <v>2031</v>
       </c>
     </row>
-    <row r="69">
-      <c r="B69" s="3" t="inlineStr">
+    <row r="70">
+      <c r="B70" s="4" t="inlineStr">
         <is>
           <t>Entry Stoops — Concrete Replacement</t>
         </is>
       </c>
-      <c r="C69" s="5" t="n">
+      <c r="C70" s="6" t="n">
         <v>196000</v>
       </c>
-      <c r="D69" s="3" t="n">
+      <c r="D70" s="4" t="n">
         <v>2032</v>
       </c>
     </row>
-    <row r="70">
-      <c r="B70" s="3" t="inlineStr">
+    <row r="71">
+      <c r="B71" s="4" t="inlineStr">
         <is>
           <t>Entry Stoops — Leveling &amp; Stair Nosing (safety)</t>
         </is>
       </c>
-      <c r="C70" s="5" t="n">
+      <c r="C71" s="6" t="n">
         <v>29400</v>
       </c>
-      <c r="D70" s="3" t="n">
+      <c r="D71" s="4" t="n">
         <v>2028</v>
       </c>
     </row>
-    <row r="71">
-      <c r="B71" s="3" t="inlineStr">
+    <row r="72">
+      <c r="B72" s="4" t="inlineStr">
         <is>
           <t>Exterior Caulk/Sealant &amp; Trim Maintenance</t>
         </is>
       </c>
-      <c r="C71" s="5" t="n">
+      <c r="C72" s="6" t="n">
         <v>15000</v>
       </c>
-      <c r="D71" s="3" t="n">
+      <c r="D72" s="4" t="n">
         <v>2027</v>
       </c>
     </row>
-    <row r="72">
-      <c r="B72" s="3" t="inlineStr">
+    <row r="73">
+      <c r="B73" s="4" t="inlineStr">
         <is>
           <t>Window Wells — rebuild program, 2027 (6 wells)</t>
         </is>
       </c>
-      <c r="C72" s="5" t="n">
+      <c r="C73" s="6" t="n">
         <v>48000</v>
       </c>
-      <c r="D72" s="3" t="n">
+      <c r="D73" s="4" t="n">
         <v>2027</v>
       </c>
     </row>
-    <row r="73">
-      <c r="B73" s="3" t="inlineStr">
+    <row r="74">
+      <c r="B74" s="4" t="inlineStr">
         <is>
           <t>Window Wells — rebuild program, 2028 (15 wells)</t>
         </is>
       </c>
-      <c r="C73" s="5" t="n">
+      <c r="C74" s="6" t="n">
         <v>120000</v>
       </c>
-      <c r="D73" s="3" t="n">
+      <c r="D74" s="4" t="n">
         <v>2028</v>
       </c>
     </row>
-    <row r="75">
-      <c r="B75" s="2" t="inlineStr">
+    <row r="76">
+      <c r="B76" s="2" t="inlineStr">
         <is>
           <t>Items NOT Included (Budget Separately)</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="B76" s="3" t="inlineStr">
+    <row r="77">
+      <c r="B77" s="4" t="inlineStr">
         <is>
           <t>The following items from the Falcon 2022 report are NOT in the Becht 2026 study and are therefore NOT included in this funding schedule. Consider budgeting for these items separately.</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="B78" s="4" t="inlineStr">
+    <row r="79">
+      <c r="B79" s="5" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="C78" s="4" t="inlineStr">
+      <c r="C79" s="5" t="inlineStr">
         <is>
           <t>Falcon Est. Cost</t>
         </is>
       </c>
-      <c r="D78" s="4" t="inlineStr">
+      <c r="D79" s="5" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="B79" s="3" t="inlineStr">
-        <is>
-          <t>Retaining Wall, Wood Tie Wells</t>
-        </is>
-      </c>
-      <c r="C79" s="5" t="n">
-        <v>15000</v>
-      </c>
-      <c r="D79" s="6" t="inlineStr">
-        <is>
-          <t>Structural/safety; Falcon estimated $15,000</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="B80" s="4" t="inlineStr">
         <is>
+          <t>Retaining Wall, Wood Tie Wells</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="n">
+        <v>15000</v>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>Structural/safety; Falcon estimated $15,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="5" t="inlineStr">
+        <is>
           <t>TOTAL OMITTED</t>
         </is>
       </c>
-      <c r="C80" s="7" t="n">
+      <c r="C81" s="7" t="n">
         <v>15000</v>
       </c>
     </row>
-    <row r="82">
-      <c r="B82" s="6" t="inlineStr">
+    <row r="83">
+      <c r="B83" s="3" t="inlineStr">
         <is>
           <t>Prepared October 2026 (re-based to 2027 to match the 2027 budget). Review and update annually.</t>
         </is>
@@ -1604,9 +1611,9 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Three decoupled funds. Yellow cells are inputs — replace placeholders with actual figures.</t>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Three decoupled funds. Yellow cells are inputs — replace placeholders with actual figures. Unaudited planning estimates; not a GAAP financial statement.</t>
         </is>
       </c>
     </row>
@@ -1618,7 +1625,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Total Reserve Cash (all accounts):</t>
         </is>
@@ -1627,14 +1634,14 @@
         <f>SUM(D12:D14)</f>
         <v/>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Auto-total of the three fund starting balances (Allocated Start column).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Number of Units:</t>
         </is>
@@ -1644,7 +1651,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Contribution Growth Rate:</t>
         </is>
@@ -1654,7 +1661,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Interest Rate on Reserves:</t>
         </is>
@@ -1777,7 +1784,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Allocated Start = each fund's current balance (yellow, editable); Total Reserve Cash (B5) is their sum. Recommended: fund near-term Long-Term Maintenance and Operating liquidity first, and build the Emergency Reserve from contributions over time.</t>
         </is>
@@ -1791,7 +1798,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Fully Funded Balance (FFB — what LTM should hold today):</t>
         </is>
@@ -1801,7 +1808,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>LTM Reserve (allocated start):</t>
         </is>
@@ -1812,7 +1819,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Percent Funded:</t>
         </is>
@@ -1821,13 +1828,13 @@
         <f>IF(B19=0,0,B20/B19)</f>
         <v/>
       </c>
-      <c r="C21" s="3">
+      <c r="C21" s="4">
         <f>IF(B21&lt;0.3,"WEAK (&lt;30% - high special-assessment risk)",IF(B21&lt;0.7,"FAIR (30-70%)","STRONG (70%+)"))</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>CAI bands: under 30% = weak; 30-70% = fair; 70%+ = strong.</t>
         </is>
@@ -1930,7 +1937,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>Combined Monthly Cost per Unit (Year 1, all three funds):</t>
         </is>
@@ -1941,14 +1948,14 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>Grows at the Growth Rate each year; this is Year-1. Add the HOA per-unit amount for a unit owner's all-in monthly.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>To model a dues reduction: lower a fund's Year-1 Contribution above and watch the status. Any target turning 'To be funded' means the reduction is not supported.</t>
         </is>
@@ -1962,7 +1969,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>Monthly Operating Expense:</t>
         </is>
@@ -1970,14 +1977,14 @@
       <c r="B37" s="9" t="n">
         <v>39286.67</v>
       </c>
-      <c r="C37" s="6" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>The association's total monthly operating spend (excludes reserve contributions).</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>Operating Reserve Multiplier (months, 1-3):</t>
         </is>
@@ -1985,7 +1992,7 @@
       <c r="B38" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="C38" s="6" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>Operating Reserve floor (row 14) = this multiplier x monthly operating expense.</t>
         </is>
@@ -2055,7 +2062,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="inlineStr">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>Equal per-unit split (fund contribution / units / 12); grows ~3%/yr. Excludes the separate $365/unit HOA dues. If common charges are set by percentage interest, larger units pay proportionally more than this average.</t>
         </is>
@@ -2140,14 +2147,14 @@
           <t>Scarborough Glen Condo Association IV — Emergency Reserve</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Floor (from Fund Summary):</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>All inputs are set on the Fund Summary sheet. This tab is calculated.</t>
         </is>
@@ -3027,7 +3034,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>All inputs are set on the Fund Summary sheet. This tab is calculated.</t>
         </is>
@@ -3899,14 +3906,14 @@
           <t>Scarborough Glen Condo Association IV — Operating Reserve</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Floor (from Fund Summary):</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>All inputs are set on the Fund Summary sheet. This tab is calculated.</t>
         </is>
@@ -4781,7 +4788,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>All costs from Becht Engineering Capital Reserve Study (2026)</t>
         </is>
@@ -5152,67 +5159,67 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>25-Year Total</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>Chimney Chase Covers</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>Deck Boards (surface)</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>Deck Framing &amp; Footings</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>Deck Railings &amp; Balusters (safety)</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>Entry Stoops — Concrete Replacement</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="K2" s="5" t="inlineStr">
         <is>
           <t>Entry Stoops — Leveling &amp; Stair Nosing (safety)</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="L2" s="5" t="inlineStr">
         <is>
           <t>Exterior Caulk/Sealant &amp; Trim Maintenance</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="M2" s="5" t="inlineStr">
         <is>
           <t>Siding, Vinyl</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="N2" s="5" t="inlineStr">
         <is>
           <t>Window Wells (rebuild program)</t>
         </is>

</xml_diff>